<commit_message>
Add 8 Korean basic vowels from Week 1 homework PDF
New vowel flashcards: 아 (a), 어 (eo), 오 (o), 우 (u), 으 (eu), 이 (i), 애 (ae), 에 (e)
Total vocabulary: 15 cards (7 words + 8 vowels)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -661,29 +661,243 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>다리</t>
+          <t>아</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>dari</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>leg / bridge</t>
+          <t>"ah" as in father</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Body / Infrastructure</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr"/>
+          <t>Vowels</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Basic vowel from Week 1 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>어</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>eo</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>"uh" as in son</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Vowels</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Basic vowel from Week 1 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>오</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>"oh" as in go</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Vowels</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Basic vowel from Week 1 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>우</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>"oo" as in moon</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Vowels</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Basic vowel from Week 1 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>으</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>eu</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>no English equivalent — unrounded, like a soft grunt</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Vowels</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Basic vowel from Week 1 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>이</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>"ee" as in see</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Vowels</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Basic vowel from Week 1 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>애</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ae</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>"ae" as in air</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Vowels</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Basic vowel from Week 1 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>에</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>"eh" as in bed</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Vowels</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Basic vowel from Week 1 homework</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 32 cards from Week 2 homework PDF
New categories:
- 10 basic consonants (ㄱ ㄴ ㄷ ㄹ ㅁ ㅂ ㅅ ㅇ ㅈ ㅎ)
- 13 compound vowels (야 여 요 유 얘 예 와 왜 외 워 웨 위 의)
- 4 aspirated consonants (ㅋ ㅌ ㅍ ㅊ)
- 5 double/tense consonants (ㄲ ㄸ ㅃ ㅆ ㅉ)
Total vocabulary: 47 cards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -875,27 +875,957 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>에</t>
+          <t>ㄱ</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>g / k</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>"eh" as in bed</t>
+          <t>"g" as in go (start) · "k" as in kite (end)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Vowels</t>
+          <t>Consonants</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Basic vowel from Week 1 homework</t>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>ㄴ</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>"n" as in no</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>ㄷ</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>d / t</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>"d" as in do (start) · "t" as in hot (end)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>ㄹ</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>r / l</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>flap between "r" and "l" — unique to Korean</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>ㅁ</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>"m" as in mom</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>ㅂ</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>b / p</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>"b" as in boy (start) · "p" as in cap (end)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>ㅅ</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>"s" as in sun</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>ㅇ</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>ng / silent</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>silent at start of syllable · "ng" as in sing at end</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>ㅈ</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>j</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>"j" as in joy</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>ㅎ</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>"h" as in hat</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Consonants</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>야</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ya</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>"ya" as in yard</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>여</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>yeo</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>"yuh" — y + eo</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>요</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>yo</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>"yo" as in yoga</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>유</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>yu</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>"yoo" as in you</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>얘</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>yae</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>"yae" — y + ae</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>ye</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>"ye" as in yes</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>와</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>wa</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>"wa" as in want</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>왜</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>wae</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>"wae" as in wax</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>외</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>oe</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>"we" — sounds like we</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>워</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>wo</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>"wuh" — w + eo</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>웨</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>we</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>"we" as in wet</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>위</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>wi</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>"wi" as in week</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>의</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>ui</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>"eui" — combination of 으 + 이</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Compound Vowels</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>ㅋ</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>k</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>aspirated "k" — strong breath puff</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Aspirated Consonants</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>ㅌ</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>aspirated "t" — strong breath puff</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Aspirated Consonants</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>ㅍ</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>aspirated "p" — strong breath puff</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Aspirated Consonants</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>ㅊ</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>ch</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>aspirated "ch" as in church</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Aspirated Consonants</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>ㄲ</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>kk</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>tense "kk" — stronger, no air puff</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>ㄸ</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>tt</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>tense "tt" — stronger, no air puff</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>ㅃ</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>tense "pp" — stronger, no air puff</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>ㅆ</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>tense "ss" — sharper than ㅅ</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>ㅉ</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>jj</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>tense "jj" — stronger, no air puff</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Week 2 homework</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 7 Batchim (받침) final consonant rules
The 7 representative batchim sounds:
ㄱ ㅋ ㄲ → K | ㄴ → N | ㄷ ㅌ ㅅ ㅆ ㅈ ㅊ ㅎ → T
ㄹ → L | ㅁ → M | ㅂ ㅍ → P | ㅇ → NG
Total vocabulary: 54 cards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1805,27 +1805,207 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>ㅉ</t>
+          <t>ㄱ ㅋ ㄲ</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>jj</t>
+          <t>K</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>tense "jj" — stronger, no air puff</t>
+          <t>Batchim sounds like K</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Double Consonants</t>
+          <t>Batchim (받침)</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Week 2 homework</t>
+          <t>Final consonant rules — @S.KAPETOKOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>ㄴ</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Batchim sounds like N</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Batchim (받침)</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Final consonant rules — @S.KAPETOKOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>ㄷ ㅌ ㅅ ㅆ ㅈ ㅊ ㅎ</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Batchim sounds like T</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Batchim (받침)</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Final consonant rules — @S.KAPETOKOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>ㄹ</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Batchim sounds like L</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Batchim (받침)</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Final consonant rules — @S.KAPETOKOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>ㅁ</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Batchim sounds like M</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Batchim (받침)</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Final consonant rules — @S.KAPETOKOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>ㅂ ㅍ</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Batchim sounds like P</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Batchim (받침)</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Final consonant rules — @S.KAPETOKOREA</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>ㅇ</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>NG</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Batchim sounds like NG</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Batchim (받침)</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>Final consonant rules — @S.KAPETOKOREA</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 4 body/speech organ vocabulary words
혀 (tongue), 입술 (lips), 이 (teeth), 목구멍 (throat)
Total vocabulary: 58 cards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1985,27 +1985,117 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>ㅇ</t>
+          <t>혀</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>hyeo</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Batchim sounds like NG</t>
+          <t>tongue</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Batchim (받침)</t>
+          <t>Body</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Final consonant rules — @S.KAPETOKOREA</t>
+          <t>Mouth/speech organs vocabulary</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>입술</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>ipsul</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>lips</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>Mouth/speech organs vocabulary</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>이</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>teeth</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>Mouth/speech organs vocabulary</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>목구멍</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>mokgumeong</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>throat</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Mouth/speech organs vocabulary</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 사자 (lion) - first Animals vocabulary
Total vocabulary: 59 cards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2098,6 +2098,32 @@
           <t>Mouth/speech organs vocabulary</t>
         </is>
       </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>사자</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>saja</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>lion</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Animals</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 자두 (plum) - Food vocabulary
Total vocabulary: 60 cards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2124,6 +2124,32 @@
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>자두</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>jadu</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>plum</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 코 (nose) - Body vocabulary
Total vocabulary: 61 cards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2150,6 +2150,32 @@
         </is>
       </c>
       <c r="F57" s="4" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>코</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>ko</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>nose</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 키 (height/stature) - Body vocabulary
Total vocabulary: 62 cards

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F58"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2176,6 +2176,36 @@
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>키</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>ki</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>height / stature</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Also means key (as in door key)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 쿠키 (cookie) and 토마토 (tomato) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,10 @@
     </font>
     <font>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Malgun Gothic"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -81,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -95,6 +99,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -460,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2206,6 +2217,58 @@
           <t>Also means key (as in door key)</t>
         </is>
       </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>쿠키</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>kuki</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>cookie</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F60" s="9" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>토마토</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>tomato</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>tomato</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F61" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 파 (green onion) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2269,6 +2269,32 @@
         </is>
       </c>
       <c r="F61" s="9" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>파</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>pa</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>green onion / scallion</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 피 (blood) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2295,6 +2295,32 @@
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>피</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>pi</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>blood</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 커피 (coffee) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2321,6 +2321,32 @@
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>커피</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>keopi</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>coffee</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 포도 (grape) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2347,6 +2347,32 @@
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>포도</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>podo</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>grape</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 차 (tea/car) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2373,6 +2373,36 @@
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>차</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>cha</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>tea / car</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>Also means car (vehicle). Context decides the meaning.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 치즈 (cheese) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2403,6 +2403,32 @@
           <t>Also means car (vehicle). Context decides the meaning.</t>
         </is>
       </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>치즈</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>chijeu</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>cheese</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 치마 (skirt) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2429,6 +2429,32 @@
         </is>
       </c>
       <c r="F67" s="7" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>치마</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>chima</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>skirt</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 포크 (fork) and 스포츠 (sports) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2455,6 +2455,58 @@
         </is>
       </c>
       <c r="F68" s="7" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>포크</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>pokeu</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>fork</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="8" t="inlineStr">
+        <is>
+          <t>스포츠</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>seupocheu</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>sports</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 피자 (pizza) and 파스타 (pasta) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2507,6 +2507,58 @@
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>피자</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>pija</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>pizza</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="8" t="inlineStr">
+        <is>
+          <t>파스타</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>paseuta</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>pasta</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 피아노 (piano) and 카페 (café) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2559,6 +2559,58 @@
         </is>
       </c>
       <c r="F72" s="7" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>피아노</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>piano</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>piano</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="7" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>카페</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>kape</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>café</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 웨이터 (waiter) and 초코 (chocolate) to vocabulary
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2611,6 +2611,62 @@
         </is>
       </c>
       <c r="F74" s="7" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>웨이터</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>weiteo</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>waiter</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="7" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="8" t="inlineStr">
+        <is>
+          <t>초코</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>choko</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>chocolate</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>Short for 초콜릿 (chokollit)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 기타 (guitar) and 카메라 (camera) to vocabulary
Words #76-77 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,10 @@
     <font>
       <name val="Malgun Gothic"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -85,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -106,6 +110,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -471,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2667,6 +2677,58 @@
           <t>Short for 초콜릿 (chokollit)</t>
         </is>
       </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="C77" s="10" t="inlineStr">
+        <is>
+          <t>gita</t>
+        </is>
+      </c>
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>guitar</t>
+        </is>
+      </c>
+      <c r="E77" s="10" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+      <c r="F77" s="10" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>카메라</t>
+        </is>
+      </c>
+      <c r="C78" s="10" t="inlineStr">
+        <is>
+          <t>kamera</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>camera</t>
+        </is>
+      </c>
+      <c r="E78" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F78" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 꼬리 (tail) to vocabulary
Word #78 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2729,6 +2729,36 @@
         </is>
       </c>
       <c r="F78" s="10" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="10" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>꼬리</t>
+        </is>
+      </c>
+      <c r="C79" s="10" t="inlineStr">
+        <is>
+          <t>kkori</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>tail</t>
+        </is>
+      </c>
+      <c r="E79" s="10" t="inlineStr">
+        <is>
+          <t>Animals</t>
+        </is>
+      </c>
+      <c r="F79" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㄲ</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 꼬마 (little kid) to vocabulary
Word #79 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2755,6 +2755,36 @@
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㄲ</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="10" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>꼬마</t>
+        </is>
+      </c>
+      <c r="C80" s="10" t="inlineStr">
+        <is>
+          <t>kkoma</t>
+        </is>
+      </c>
+      <c r="D80" s="10" t="inlineStr">
+        <is>
+          <t>little kid / toddler</t>
+        </is>
+      </c>
+      <c r="E80" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F80" s="10" t="inlineStr">
         <is>
           <t>Double consonant ㄲ</t>
         </is>

</xml_diff>

<commit_message>
Add 쌀 (rice) to vocabulary
Word #80 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2787,6 +2787,36 @@
       <c r="F80" s="10" t="inlineStr">
         <is>
           <t>Double consonant ㄲ</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="10" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>쌀</t>
+        </is>
+      </c>
+      <c r="C81" s="10" t="inlineStr">
+        <is>
+          <t>ssal</t>
+        </is>
+      </c>
+      <c r="D81" s="10" t="inlineStr">
+        <is>
+          <t>rice (uncooked)</t>
+        </is>
+      </c>
+      <c r="E81" s="10" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F81" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅆ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 또 (again/also) and 다시 (again/once more) to vocabulary
Words #81-82 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2819,6 +2819,62 @@
           <t>Double consonant ㅆ</t>
         </is>
       </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="10" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>또</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>tto</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>again / also</t>
+        </is>
+      </c>
+      <c r="E82" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㄸ</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="11" t="inlineStr">
+        <is>
+          <t>다시</t>
+        </is>
+      </c>
+      <c r="C83" s="10" t="inlineStr">
+        <is>
+          <t>dasi</t>
+        </is>
+      </c>
+      <c r="D83" s="10" t="inlineStr">
+        <is>
+          <t>again / once more</t>
+        </is>
+      </c>
+      <c r="E83" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F83" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 허리띠 (belt) to vocabulary
Word #83 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2875,6 +2875,36 @@
         </is>
       </c>
       <c r="F83" s="10" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="10" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>허리띠</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>heoritti</t>
+        </is>
+      </c>
+      <c r="D84" s="10" t="inlineStr">
+        <is>
+          <t>belt</t>
+        </is>
+      </c>
+      <c r="E84" s="10" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="F84" s="10" t="inlineStr">
+        <is>
+          <t>허리 (waist) + 띠 (band)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 아빠 (dad) to vocabulary
Word #84 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2903,6 +2903,36 @@
       <c r="F84" s="10" t="inlineStr">
         <is>
           <t>허리 (waist) + 띠 (band)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="10" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>아빠</t>
+        </is>
+      </c>
+      <c r="C85" s="10" t="inlineStr">
+        <is>
+          <t>appa</t>
+        </is>
+      </c>
+      <c r="D85" s="10" t="inlineStr">
+        <is>
+          <t>dad / daddy</t>
+        </is>
+      </c>
+      <c r="E85" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F85" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅃ; informal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 오빠 (older brother) to vocabulary
Word #85 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F85"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2933,6 +2933,36 @@
       <c r="F85" s="10" t="inlineStr">
         <is>
           <t>Double consonant ㅃ; informal</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>오빠</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>oppa</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>older brother (used by females)</t>
+        </is>
+      </c>
+      <c r="E86" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F86" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅃ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add close family vocabulary (#86-100)
15 family words: 엄마, 아버지, 어머니, 형, 누나, 언니, 남동생, 여동생,
할아버지, 할머니, 아들, 딸, 남편, 아내, 가족

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2965,6 +2965,408 @@
           <t>Double consonant ㅃ</t>
         </is>
       </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="10" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>엄마</t>
+        </is>
+      </c>
+      <c r="C87" s="10" t="inlineStr">
+        <is>
+          <t>eomma</t>
+        </is>
+      </c>
+      <c r="D87" s="10" t="inlineStr">
+        <is>
+          <t>mom / mommy</t>
+        </is>
+      </c>
+      <c r="E87" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F87" s="10" t="inlineStr">
+        <is>
+          <t>informal</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="11" t="inlineStr">
+        <is>
+          <t>아버지</t>
+        </is>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>abeoji</t>
+        </is>
+      </c>
+      <c r="D88" s="10" t="inlineStr">
+        <is>
+          <t>father</t>
+        </is>
+      </c>
+      <c r="E88" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F88" s="10" t="inlineStr">
+        <is>
+          <t>formal/respectful</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="10" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="11" t="inlineStr">
+        <is>
+          <t>어머니</t>
+        </is>
+      </c>
+      <c r="C89" s="10" t="inlineStr">
+        <is>
+          <t>eomeoni</t>
+        </is>
+      </c>
+      <c r="D89" s="10" t="inlineStr">
+        <is>
+          <t>mother</t>
+        </is>
+      </c>
+      <c r="E89" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F89" s="10" t="inlineStr">
+        <is>
+          <t>formal/respectful</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>형</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>hyeong</t>
+        </is>
+      </c>
+      <c r="D90" s="10" t="inlineStr">
+        <is>
+          <t>older brother (used by males)</t>
+        </is>
+      </c>
+      <c r="E90" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F90" s="10" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="11" t="inlineStr">
+        <is>
+          <t>누나</t>
+        </is>
+      </c>
+      <c r="C91" s="10" t="inlineStr">
+        <is>
+          <t>nuna</t>
+        </is>
+      </c>
+      <c r="D91" s="10" t="inlineStr">
+        <is>
+          <t>older sister (used by males)</t>
+        </is>
+      </c>
+      <c r="E91" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F91" s="10" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="11" t="inlineStr">
+        <is>
+          <t>언니</t>
+        </is>
+      </c>
+      <c r="C92" s="10" t="inlineStr">
+        <is>
+          <t>eonni</t>
+        </is>
+      </c>
+      <c r="D92" s="10" t="inlineStr">
+        <is>
+          <t>older sister (used by females)</t>
+        </is>
+      </c>
+      <c r="E92" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F92" s="10" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="11" t="inlineStr">
+        <is>
+          <t>남동생</t>
+        </is>
+      </c>
+      <c r="C93" s="10" t="inlineStr">
+        <is>
+          <t>namdongsaeng</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="inlineStr">
+        <is>
+          <t>younger brother</t>
+        </is>
+      </c>
+      <c r="E93" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F93" s="10" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="10" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>여동생</t>
+        </is>
+      </c>
+      <c r="C94" s="10" t="inlineStr">
+        <is>
+          <t>yeodongsaeng</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="inlineStr">
+        <is>
+          <t>younger sister</t>
+        </is>
+      </c>
+      <c r="E94" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F94" s="10" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="11" t="inlineStr">
+        <is>
+          <t>할아버지</t>
+        </is>
+      </c>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>harabeoji</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="inlineStr">
+        <is>
+          <t>grandfather</t>
+        </is>
+      </c>
+      <c r="E95" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F95" s="10" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="11" t="inlineStr">
+        <is>
+          <t>할머니</t>
+        </is>
+      </c>
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>halmeoni</t>
+        </is>
+      </c>
+      <c r="D96" s="10" t="inlineStr">
+        <is>
+          <t>grandmother</t>
+        </is>
+      </c>
+      <c r="E96" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F96" s="10" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="11" t="inlineStr">
+        <is>
+          <t>아들</t>
+        </is>
+      </c>
+      <c r="C97" s="10" t="inlineStr">
+        <is>
+          <t>adeul</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="inlineStr">
+        <is>
+          <t>son</t>
+        </is>
+      </c>
+      <c r="E97" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F97" s="10" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="10" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>딸</t>
+        </is>
+      </c>
+      <c r="C98" s="10" t="inlineStr">
+        <is>
+          <t>ttal</t>
+        </is>
+      </c>
+      <c r="D98" s="10" t="inlineStr">
+        <is>
+          <t>daughter</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F98" s="10" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="11" t="inlineStr">
+        <is>
+          <t>남편</t>
+        </is>
+      </c>
+      <c r="C99" s="10" t="inlineStr">
+        <is>
+          <t>nampyeon</t>
+        </is>
+      </c>
+      <c r="D99" s="10" t="inlineStr">
+        <is>
+          <t>husband</t>
+        </is>
+      </c>
+      <c r="E99" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F99" s="10" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>아내</t>
+        </is>
+      </c>
+      <c r="C100" s="10" t="inlineStr">
+        <is>
+          <t>anae</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>wife</t>
+        </is>
+      </c>
+      <c r="E100" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F100" s="10" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>가족</t>
+        </is>
+      </c>
+      <c r="C101" s="10" t="inlineStr">
+        <is>
+          <t>gajok</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="E101" s="10" t="inlineStr">
+        <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="F101" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 빨리 (quickly/hurry) to vocabulary
Word #101 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3367,6 +3367,36 @@
         </is>
       </c>
       <c r="F101" s="10" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="10" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>빨리</t>
+        </is>
+      </c>
+      <c r="C102" s="10" t="inlineStr">
+        <is>
+          <t>ppalli</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>quickly / hurry</t>
+        </is>
+      </c>
+      <c r="E102" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F102" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅃ; adverb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 뿔 (horn) to vocabulary
Word #102 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3395,6 +3395,36 @@
       <c r="F102" s="10" t="inlineStr">
         <is>
           <t>Double consonant ㅃ; adverb</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
+          <t>뿔</t>
+        </is>
+      </c>
+      <c r="C103" s="10" t="inlineStr">
+        <is>
+          <t>ppul</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="inlineStr">
+        <is>
+          <t>horn</t>
+        </is>
+      </c>
+      <c r="E103" s="10" t="inlineStr">
+        <is>
+          <t>Animals</t>
+        </is>
+      </c>
+      <c r="F103" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅃ; batchim ㄹ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct card #102: 뿔 (horn) → 뼈 (bone)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -3404,27 +3404,27 @@
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>뿔</t>
+          <t>뼈</t>
         </is>
       </c>
       <c r="C103" s="10" t="inlineStr">
         <is>
-          <t>ppul</t>
+          <t>ppyeo</t>
         </is>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>horn</t>
+          <t>bone</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>Animals</t>
+          <t>Body</t>
         </is>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>Double consonant ㅃ; batchim ㄹ</t>
+          <t>Double consonant ㅃ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 싸요 (cheap) and 비싸요 (expensive) to vocabulary
Words #103-104 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3425,6 +3425,66 @@
       <c r="F103" s="10" t="inlineStr">
         <is>
           <t>Double consonant ㅃ</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="10" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="11" t="inlineStr">
+        <is>
+          <t>싸요</t>
+        </is>
+      </c>
+      <c r="C104" s="10" t="inlineStr">
+        <is>
+          <t>ssayo</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="inlineStr">
+        <is>
+          <t>cheap / inexpensive</t>
+        </is>
+      </c>
+      <c r="E104" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F104" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅆ; polite form of 싸다</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>비싸요</t>
+        </is>
+      </c>
+      <c r="C105" s="10" t="inlineStr">
+        <is>
+          <t>bissayo</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="inlineStr">
+        <is>
+          <t>expensive</t>
+        </is>
+      </c>
+      <c r="E105" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F105" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅆ; polite form of 비싸다</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 쓰레기 (trash/garbage) to vocabulary
Word #105 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3485,6 +3485,36 @@
       <c r="F105" s="10" t="inlineStr">
         <is>
           <t>Double consonant ㅆ; polite form of 비싸다</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="10" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>쓰레기</t>
+        </is>
+      </c>
+      <c r="C106" s="10" t="inlineStr">
+        <is>
+          <t>sseuregi</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="inlineStr">
+        <is>
+          <t>trash / garbage</t>
+        </is>
+      </c>
+      <c r="E106" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F106" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅆ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 찌개 (stew) to vocabulary
Word #106 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3515,6 +3515,36 @@
       <c r="F106" s="10" t="inlineStr">
         <is>
           <t>Double consonant ㅆ</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>찌개</t>
+        </is>
+      </c>
+      <c r="C107" s="10" t="inlineStr">
+        <is>
+          <t>jjigae</t>
+        </is>
+      </c>
+      <c r="D107" s="10" t="inlineStr">
+        <is>
+          <t>stew</t>
+        </is>
+      </c>
+      <c r="E107" s="10" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F107" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㅉ; e.g. 김치찌개</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 5 double consonants (ㄲ, ㄸ, ㅃ, ㅆ, ㅉ) as reference cards
Cards #107-111 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3545,6 +3545,156 @@
       <c r="F107" s="10" t="inlineStr">
         <is>
           <t>Double consonant ㅉ; e.g. 김치찌개</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="10" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>ㄲ</t>
+        </is>
+      </c>
+      <c r="C108" s="10" t="inlineStr">
+        <is>
+          <t>kk</t>
+        </is>
+      </c>
+      <c r="D108" s="10" t="inlineStr">
+        <is>
+          <t>double ㄱ (ssang-giyeok)</t>
+        </is>
+      </c>
+      <c r="E108" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F108" s="10" t="inlineStr">
+        <is>
+          <t>까, 꼬, 끼</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>ㄸ</t>
+        </is>
+      </c>
+      <c r="C109" s="10" t="inlineStr">
+        <is>
+          <t>tt</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="inlineStr">
+        <is>
+          <t>double ㄷ (ssang-digeut)</t>
+        </is>
+      </c>
+      <c r="E109" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F109" s="10" t="inlineStr">
+        <is>
+          <t>따, 또, 띠</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="10" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="11" t="inlineStr">
+        <is>
+          <t>ㅃ</t>
+        </is>
+      </c>
+      <c r="C110" s="10" t="inlineStr">
+        <is>
+          <t>pp</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="inlineStr">
+        <is>
+          <t>double ㅂ (ssang-bieup)</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F110" s="10" t="inlineStr">
+        <is>
+          <t>빠, 뽀, 삐</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
+          <t>ㅆ</t>
+        </is>
+      </c>
+      <c r="C111" s="10" t="inlineStr">
+        <is>
+          <t>ss</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="inlineStr">
+        <is>
+          <t>double ㅅ (ssang-siot)</t>
+        </is>
+      </c>
+      <c r="E111" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F111" s="10" t="inlineStr">
+        <is>
+          <t>싸, 쏘, 씨</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="10" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>ㅉ</t>
+        </is>
+      </c>
+      <c r="C112" s="10" t="inlineStr">
+        <is>
+          <t>jj</t>
+        </is>
+      </c>
+      <c r="D112" s="10" t="inlineStr">
+        <is>
+          <t>double ㅈ (ssang-jieut)</t>
+        </is>
+      </c>
+      <c r="E112" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F112" s="10" t="inlineStr">
+        <is>
+          <t>짜, 쪼, 찌</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 15 double consonant practice syllables (#112-126)
까꼬끼, 따또띠, 빠뽀삐, 싸쏘씨, 짜쪼찌 with example words.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F112"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3695,6 +3695,456 @@
       <c r="F112" s="10" t="inlineStr">
         <is>
           <t>짜, 쪼, 찌</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>까</t>
+        </is>
+      </c>
+      <c r="C113" s="10" t="inlineStr">
+        <is>
+          <t>kka</t>
+        </is>
+      </c>
+      <c r="D113" s="10" t="inlineStr">
+        <is>
+          <t>syllable (kka)</t>
+        </is>
+      </c>
+      <c r="E113" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F113" s="10" t="inlineStr">
+        <is>
+          <t>ㄲ + ㅏ</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="10" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="11" t="inlineStr">
+        <is>
+          <t>꼬</t>
+        </is>
+      </c>
+      <c r="C114" s="10" t="inlineStr">
+        <is>
+          <t>kko</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="inlineStr">
+        <is>
+          <t>syllable (kko)</t>
+        </is>
+      </c>
+      <c r="E114" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F114" s="10" t="inlineStr">
+        <is>
+          <t>ㄲ + ㅗ; e.g. 꼬리 (tail)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>끼</t>
+        </is>
+      </c>
+      <c r="C115" s="10" t="inlineStr">
+        <is>
+          <t>kki</t>
+        </is>
+      </c>
+      <c r="D115" s="10" t="inlineStr">
+        <is>
+          <t>syllable (kki)</t>
+        </is>
+      </c>
+      <c r="E115" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F115" s="10" t="inlineStr">
+        <is>
+          <t>ㄲ + ㅣ; e.g. 끼니 (meal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="10" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>따</t>
+        </is>
+      </c>
+      <c r="C116" s="10" t="inlineStr">
+        <is>
+          <t>tta</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="inlineStr">
+        <is>
+          <t>syllable (tta)</t>
+        </is>
+      </c>
+      <c r="E116" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F116" s="10" t="inlineStr">
+        <is>
+          <t>ㄸ + ㅏ; e.g. 따뜻하다 (warm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="10" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>또</t>
+        </is>
+      </c>
+      <c r="C117" s="10" t="inlineStr">
+        <is>
+          <t>tto</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="inlineStr">
+        <is>
+          <t>syllable (tto)</t>
+        </is>
+      </c>
+      <c r="E117" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F117" s="10" t="inlineStr">
+        <is>
+          <t>ㄸ + ㅗ; also = again</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="11" t="inlineStr">
+        <is>
+          <t>띠</t>
+        </is>
+      </c>
+      <c r="C118" s="10" t="inlineStr">
+        <is>
+          <t>tti</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="inlineStr">
+        <is>
+          <t>syllable (tti)</t>
+        </is>
+      </c>
+      <c r="E118" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F118" s="10" t="inlineStr">
+        <is>
+          <t>ㄸ + ㅣ; e.g. 허리띠 (belt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>빠</t>
+        </is>
+      </c>
+      <c r="C119" s="10" t="inlineStr">
+        <is>
+          <t>ppa</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="inlineStr">
+        <is>
+          <t>syllable (ppa)</t>
+        </is>
+      </c>
+      <c r="E119" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F119" s="10" t="inlineStr">
+        <is>
+          <t>ㅃ + ㅏ; e.g. 아빠 (dad)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>뽀</t>
+        </is>
+      </c>
+      <c r="C120" s="10" t="inlineStr">
+        <is>
+          <t>ppo</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="inlineStr">
+        <is>
+          <t>syllable (ppo)</t>
+        </is>
+      </c>
+      <c r="E120" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F120" s="10" t="inlineStr">
+        <is>
+          <t>ㅃ + ㅗ; e.g. 뽀뽀 (kiss)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="10" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>삐</t>
+        </is>
+      </c>
+      <c r="C121" s="10" t="inlineStr">
+        <is>
+          <t>ppi</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="inlineStr">
+        <is>
+          <t>syllable (ppi)</t>
+        </is>
+      </c>
+      <c r="E121" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F121" s="10" t="inlineStr">
+        <is>
+          <t>ㅃ + ㅣ; e.g. 삐지다 (sulk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="10" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>싸</t>
+        </is>
+      </c>
+      <c r="C122" s="10" t="inlineStr">
+        <is>
+          <t>ssa</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="inlineStr">
+        <is>
+          <t>syllable (ssa)</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F122" s="10" t="inlineStr">
+        <is>
+          <t>ㅆ + ㅏ; e.g. 싸요 (cheap)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>쏘</t>
+        </is>
+      </c>
+      <c r="C123" s="10" t="inlineStr">
+        <is>
+          <t>sso</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>syllable (sso)</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
+          <t>ㅆ + ㅗ; e.g. 쏘다 (shoot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>씨</t>
+        </is>
+      </c>
+      <c r="C124" s="10" t="inlineStr">
+        <is>
+          <t>ssi</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>Mr./Ms. (honorific)</t>
+        </is>
+      </c>
+      <c r="E124" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F124" s="10" t="inlineStr">
+        <is>
+          <t>ㅆ + ㅣ; e.g. 김씨 (Mr./Ms. Kim)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>짜</t>
+        </is>
+      </c>
+      <c r="C125" s="10" t="inlineStr">
+        <is>
+          <t>jja</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>salty / to squeeze</t>
+        </is>
+      </c>
+      <c r="E125" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F125" s="10" t="inlineStr">
+        <is>
+          <t>ㅉ + ㅏ; 짜다 = salty</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>쪼</t>
+        </is>
+      </c>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>jjo</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>syllable (jjo)</t>
+        </is>
+      </c>
+      <c r="E126" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F126" s="10" t="inlineStr">
+        <is>
+          <t>ㅉ + ㅗ; e.g. 쪼개다 (split)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>찌</t>
+        </is>
+      </c>
+      <c r="C127" s="10" t="inlineStr">
+        <is>
+          <t>jji</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t>syllable (jji)</t>
+        </is>
+      </c>
+      <c r="E127" s="10" t="inlineStr">
+        <is>
+          <t>Double Consonants</t>
+        </is>
+      </c>
+      <c r="F127" s="10" t="inlineStr">
+        <is>
+          <t>ㅉ + ㅣ; e.g. 찌개 (stew)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 하늘 (sky), 땅 (earth), 사람 (people) to vocabulary
Words #127-129: the 3 core concepts of Korean philosophy.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4145,6 +4145,96 @@
       <c r="F127" s="10" t="inlineStr">
         <is>
           <t>ㅉ + ㅣ; e.g. 찌개 (stew)</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="11" t="inlineStr">
+        <is>
+          <t>하늘</t>
+        </is>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>haneul</t>
+        </is>
+      </c>
+      <c r="D128" s="10" t="inlineStr">
+        <is>
+          <t>sky / heaven / spirit</t>
+        </is>
+      </c>
+      <c r="E128" s="10" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="F128" s="10" t="inlineStr">
+        <is>
+          <t>One of the 3 core concepts: 하늘, 땅, 사람</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>땅</t>
+        </is>
+      </c>
+      <c r="C129" s="10" t="inlineStr">
+        <is>
+          <t>ttang</t>
+        </is>
+      </c>
+      <c r="D129" s="10" t="inlineStr">
+        <is>
+          <t>earth / ground / real world</t>
+        </is>
+      </c>
+      <c r="E129" s="10" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="F129" s="10" t="inlineStr">
+        <is>
+          <t>Double consonant ㄸ; one of 하늘, 땅, 사람</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="11" t="inlineStr">
+        <is>
+          <t>사람</t>
+        </is>
+      </c>
+      <c r="C130" s="10" t="inlineStr">
+        <is>
+          <t>saram</t>
+        </is>
+      </c>
+      <c r="D130" s="10" t="inlineStr">
+        <is>
+          <t>people / person</t>
+        </is>
+      </c>
+      <c r="E130" s="10" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F130" s="10" t="inlineStr">
+        <is>
+          <t>One of the 3 core concepts: 하늘, 땅, 사람</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 우유 (milk) and 여우 (fox) to vocabulary
Words #130-131 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F130"/>
+  <dimension ref="A1:F132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4237,6 +4237,58 @@
           <t>One of the 3 core concepts: 하늘, 땅, 사람</t>
         </is>
       </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>우유</t>
+        </is>
+      </c>
+      <c r="C131" s="10" t="inlineStr">
+        <is>
+          <t>uyu</t>
+        </is>
+      </c>
+      <c r="D131" s="10" t="inlineStr">
+        <is>
+          <t>milk</t>
+        </is>
+      </c>
+      <c r="E131" s="10" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F131" s="10" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="10" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="11" t="inlineStr">
+        <is>
+          <t>여우</t>
+        </is>
+      </c>
+      <c r="C132" s="10" t="inlineStr">
+        <is>
+          <t>yeou</t>
+        </is>
+      </c>
+      <c r="D132" s="10" t="inlineStr">
+        <is>
+          <t>fox</t>
+        </is>
+      </c>
+      <c r="E132" s="10" t="inlineStr">
+        <is>
+          <t>Animals</t>
+        </is>
+      </c>
+      <c r="F132" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 머리 (head/hair) to vocabulary
Word #132 added to Excel file and flashcard database.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F132"/>
+  <dimension ref="A1:F133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4289,6 +4289,32 @@
         </is>
       </c>
       <c r="F132" s="10" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
+          <t>머리</t>
+        </is>
+      </c>
+      <c r="C133" s="10" t="inlineStr">
+        <is>
+          <t>meori</t>
+        </is>
+      </c>
+      <c r="D133" s="10" t="inlineStr">
+        <is>
+          <t>head / hair</t>
+        </is>
+      </c>
+      <c r="E133" s="10" t="inlineStr">
+        <is>
+          <t>Body</t>
+        </is>
+      </c>
+      <c r="F133" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 142 Sejong Korean 1A vocabulary entries (ISBN 978-1-63519-043-4)
Import vocabulary from 세종한국어 1A (Sejong Korean 1A) textbook covering:
- Greetings & basic phrases (10 entries)
- Self-introduction & occupations (8 entries)
- Countries (7 entries)
- Objects & classroom items (11 entries)
- Food & drink (7 entries)
- Numbers: native Korean 1-10 & Sino-Korean 1-10,000 (24 entries)
- Places (12 entries)
- Verbs (21 entries)
- Time & days of the week (19 entries)
- Weather (4 entries)
- Adjectives (6 entries)
- Transportation (4 entries)
- Question words (7 entries)
- Activities (2 entries)

Total vocabulary now: 274 entries (132 existing + 142 Sejong 1A)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vcc9Bzf8Kbtj4Cyv9aE2G1
</commit_message>
<xml_diff>
--- a/korean_vocabulary.xlsx
+++ b/korean_vocabulary.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4315,6 +4315,4266 @@
         </is>
       </c>
       <c r="F133" s="10" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>134</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>안녕하세요</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>annyeonghaseyo</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>hello (formal)</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 1 · Most common greeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>135</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>감사합니다</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>gamsahamnida</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>thank you (formal)</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>136</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>죄송합니다</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>joesonghamnida</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>I'm sorry (formal)</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>137</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>네</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 1 · Also written 예 (ye)</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>138</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>아니요</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>aniyo</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>139</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>만나서 반갑습니다</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>mannaseo bangapseumnida</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>nice to meet you</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>140</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>안녕히 가세요</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>annyeonghi gaseyo</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>goodbye (to someone leaving)</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 1 · Said by the one staying</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>141</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>안녕히 계세요</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>annyeonghi gyeseyo</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>goodbye (to someone staying)</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 1 · Said by the one leaving</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>142</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>주세요</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>juseyo</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>please give me</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · 물 주세요 = Water, please</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>143</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>알겠습니다</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>algesseumnida</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>I understand</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Greetings</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Sejong 1A · Very formal</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>144</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>저</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>jeo</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>I (humble/formal)</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2 · Humble form; casual = 나 (na)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>145</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>이름</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>ireum</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>146</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>학생</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>haksaeng</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>student</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>147</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>선생님</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>seonsaengnim</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>teacher (honorific)</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2 · -님 is honorific suffix</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>148</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>회사원</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>hoesawon</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>office worker</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>149</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>의사</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>uisa</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>doctor</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>150</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>친구</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>chingu</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>friend</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>151</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>전화번호</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>jeonhwabeonho</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>phone number</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>152</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>한국</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>hanguk</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Korea</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Countries</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2 · 한국 사람 = Korean person</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>153</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>일본</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>ilbon</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Countries</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>154</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>중국</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>jungguk</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Countries</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>155</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>미국</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>miguk</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>America / USA</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Countries</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>156</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>베트남</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>beteunam</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Countries</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>157</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>태국</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>taeguk</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Thailand</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Countries</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>158</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>독일</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>dogil</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Countries</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>159</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>책</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>chaek</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>160</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>가방</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>gabang</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>bag</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>161</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>연필</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>yeonpil</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>pencil</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>162</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>지우개</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>jiugae</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>eraser</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>163</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>컴퓨터</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>keompyuteo</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>computer</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>164</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>휴대폰</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>hyudaepon</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>cell phone</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · Also 핸드폰</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>165</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>시계</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>sigye</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>clock / watch</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>166</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>우산</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>usan</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>umbrella</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>167</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>의자</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>uija</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>chair</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>168</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>책상</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>chaeksang</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>desk</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · 책 (book) + 상 (table)</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>169</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>사전</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>sajeon</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>dictionary</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Objects</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>170</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>물</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>mul</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>171</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>빵</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>ppang</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>bread</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5 · Double consonant ㅃ</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>172</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>밥</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>bap</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>rice (cooked) / meal</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5 · Batchim ㅂ→P</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>173</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>한식</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>hansik</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Korean food</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5 · 한 (Korean) + 식 (food)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>174</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>과일</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>gwail</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>fruit</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>175</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>고기</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>gogi</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>meat</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>176</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>야채</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>yachae</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>vegetable</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5 · Also 채소 (chaeso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>177</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>하나</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>hana</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>one (native Korean)</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · Used for counting items</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>178</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>둘</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>dul</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>two (native Korean)</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>179</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>셋</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>three (native Korean)</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>180</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>넷</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>net</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>four (native Korean)</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>181</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>다섯</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>daseot</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>five (native Korean)</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>182</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>여섯</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>yeoseot</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>six (native Korean)</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>183</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>일곱</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>ilgop</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>seven (native Korean)</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>184</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>여덟</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>yeodeol</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>eight (native Korean)</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>185</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>아홉</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>ahop</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>nine (native Korean)</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>186</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>열</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>yeol</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>ten (native Korean)</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>187</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>일</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>il</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>one (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · Used for dates, money, phone #s</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>188</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>이</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>two (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · Context: 이 as number, not teeth</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>189</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>삼</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>sam</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>three (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>190</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>사</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>sa</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>four (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>191</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>오</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>five (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>192</v>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>육</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>yuk</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>six (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>193</v>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>칠</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>chil</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>seven (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>194</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>팔</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>pal</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>eight (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>195</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>구</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>gu</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>nine (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>196</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>십</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>sip</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>ten (Sino-Korean)</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>197</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>백</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>baek</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>hundred</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · Sino-Korean</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>198</v>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>천</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>cheon</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>thousand</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · Sino-Korean</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>199</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>만</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>man</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>ten thousand</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · Sino-Korean; 10,000 is a key unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>200</v>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>원</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>won</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>won (Korean currency)</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Numbers</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · 이천 원 = 2,000 won</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>201</v>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>학교</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>hakgyo</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>school</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>202</v>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>회사</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>hoesa</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>company / office</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>203</v>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>집</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>jip</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>house / home</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · Batchim ㅂ→P</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>204</v>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>가게</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>gage</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>store / shop</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>205</v>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>sijang</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>market</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>206</v>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>식당</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>sikdang</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>207</v>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>은행</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>eunhaeng</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>bank</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>208</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>병원</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>byeongwon</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>209</v>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>약국</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>yakguk</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>pharmacy</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>210</v>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>도서관</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>doseogwan</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>library</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>211</v>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>공원</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>gongwon</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>park</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>212</v>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>편의점</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>pyeonuijeom</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>convenience store</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>213</v>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>가다</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>gada</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>to go</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · 가요 (polite form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>214</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>오다</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>oda</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>to come</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · 와요 (polite form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>215</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>먹다</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>meokda</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>to eat</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5 · 먹어요 (polite form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>216</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>마시다</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>masida</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>to drink</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5 · 마셔요 (polite form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>217</v>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>보다</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>boda</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>to see / to watch</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 봐요 (polite form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>218</v>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>읽다</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>ikda</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>to read</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 읽어요; batchim ㄹㄱ→K</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>219</v>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>쓰다</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>sseuda</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>to write / to use</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · Double ㅆ; 써요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>220</v>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>듣다</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>deutda</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>to listen / to hear</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · Irregular: 들어요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>221</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>말하다</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>malhada</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>to speak / to talk</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2 · 말해요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>222</v>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>배우다</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>baeuda</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>to learn</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 배워요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>223</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>사다</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>sada</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>to buy</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · 사요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>224</v>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>있다</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>itda</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>to exist / to have</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · 있어요 (polite); opposite: 없다</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>225</v>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>없다</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>eopda</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>to not exist / to not have</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · 없어요 (polite); opposite: 있다</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>226</v>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>하다</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>hada</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>to do</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6 · 해요 (polite); very versatile verb</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>227</v>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>자다</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>jada</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>to sleep</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6 · 자요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>228</v>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>일어나다</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>ireonada</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>to get up / to wake up</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6 · 일어나요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>229</v>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>공부하다</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>gongbuhada</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>to study</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6 · 공부해요 (polite); 공부 = study</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>230</v>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>운동하다</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>undonghada</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>to exercise</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 운동해요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>231</v>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>좋다</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>jota</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>to be good / to like</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 좋아요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>232</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>만나다</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>mannada</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>to meet</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 만나요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>233</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>요리하다</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>yorihada</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>to cook</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 요리해요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>234</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>시</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>si</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>o'clock / hour</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6 · 두 시 = 2 o'clock (native numbers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>235</v>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>분</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>bun</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>minute</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6 · 삼십 분 = 30 min (Sino numbers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>236</v>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>오전</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>ojeon</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>AM / morning</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>237</v>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>오후</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>ohu</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>PM / afternoon</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>238</v>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>아침</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>achim</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>morning / breakfast</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6 · Also means breakfast</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>239</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>점심</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>jeomsim</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>lunch</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>240</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>저녁</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>jeonyeok</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>evening / dinner</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6 · Also means dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>241</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>지금</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>jigeum</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>now</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>242</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>오늘</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>oneul</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>today</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>243</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>내일</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>naeil</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>tomorrow</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>244</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>어제</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>eoje</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>yesterday</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>245</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>월요일</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>woryoil</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 월 = moon/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>246</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>화요일</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>hwayoil</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 화 = fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>247</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>수요일</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>suyoil</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 수 = water</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>248</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>목요일</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>mogyoil</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 목 = wood</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>249</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>금요일</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>geumyoil</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 금 = gold/metal</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>250</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>토요일</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>toyoil</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Saturday</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 토 = earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>251</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>일요일</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>iryoil</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Sunday</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 일 = sun/day</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>252</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>주말</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>jumal</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 주 (week) + 말 (end)</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>253</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>날씨</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>nalssi</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8 · Double ㅆ</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>254</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>비</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>bi</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>rain</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8 · 비가 와요 = It's raining</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>255</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>눈</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>nun</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>snow / eye</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8 · Two meanings: snow + eye</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>256</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>바람</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>baram</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>wind</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Weather</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>257</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>크다</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>keuda</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>to be big</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Adjectives</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · 커요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>258</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>작다</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>jakda</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>to be small</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Adjectives</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · 작아요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>259</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>많다</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>manta</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>to be many / much</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Adjectives</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · 많아요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>260</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>맛있다</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>masitda</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>to be delicious</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Adjectives</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 5 · 맛있어요 (polite); 맛 = taste</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>261</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>덥다</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>deopda</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>to be hot (weather)</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Adjectives</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8 · Irregular: 더워요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>262</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>춥다</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>chupda</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>to be cold (weather)</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Adjectives</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8 · Irregular: 추워요 (polite)</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>263</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>버스</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>beoseu</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>264</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>지하철</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>jihacheol</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>subway</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8 · 지하 (underground) + 철 (iron)</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>265</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>택시</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>taeksi</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>taxi</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>266</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>자전거</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>jajeongeo</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>bicycle</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>267</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>뭐</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>mwo</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>what</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Question Words</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3 · Also 무엇 (formal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>268</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>어디</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>eodi</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>where</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Question Words</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>269</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>누구</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>nugu</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>who</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Question Words</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>270</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>언제</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>eonje</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>when</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Question Words</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>271</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>왜</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>wae</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>why</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Question Words</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>272</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>어떻게</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>eotteoke</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>how</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Question Words</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>273</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>얼마</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>eolma</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>how much</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Question Words</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 4 · 얼마예요? = How much is it?</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>274</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>영화</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>yeonghwa</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>movie</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 영화를 봐요 = I watch a movie</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>275</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>음악</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>eumak</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>music</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Activities</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Sejong 1A Unit 7 · 음악을 들어요 = I listen to music</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>